<commit_message>
feat(2026): mise a niveau Cartino2D unifiee, templates assainis, exemples C2D_ParamUser, securisation acces et gitignore
</commit_message>
<xml_diff>
--- a/PreC2D/Data_PluieRaster.xlsx
+++ b/PreC2D/Data_PluieRaster.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R\R-4.4.1\Cerema\PreC2D\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38844034-A8C3-4196-BDE5-D4303564A6F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C20D79-0559-4788-8E67-CC963AC2D1E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -26,12 +26,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="135">
   <si>
     <t>Cas</t>
   </si>
@@ -93,12 +96,18 @@
     <t>TypPluie</t>
   </si>
   <si>
+    <t>Formatdate</t>
+  </si>
+  <si>
     <t>Boris</t>
   </si>
   <si>
     <t>Fred</t>
   </si>
   <si>
+    <t>Nabil</t>
+  </si>
+  <si>
     <t>Anti</t>
   </si>
   <si>
@@ -159,6 +168,9 @@
     <t>D:\PICS\FTP\envoiMF09062021\05_Antilope_1h_J+1</t>
   </si>
   <si>
+    <t>E:\Pluie\PICS\envoiMF09062021\05_Antilope_1h_J+1</t>
+  </si>
+  <si>
     <t>J4</t>
   </si>
   <si>
@@ -168,6 +180,9 @@
     <t>D:\PICS\FTP\envoiMF09062021\03_Antilope_15min_Tdiff</t>
   </si>
   <si>
+    <t>E:\Pluie\PICS\envoiMF09062021\03_Antilope_15min_Tdiff</t>
+  </si>
+  <si>
     <t>J5</t>
   </si>
   <si>
@@ -183,6 +198,9 @@
     <t>D:\PICS\FTP\envoiMF09062021\08_Antilope_15min_Tdiff_inter</t>
   </si>
   <si>
+    <t>E:\Pluie\PICS\envoiMF09062021\08_Antilope_15min_Tdiff_inter</t>
+  </si>
+  <si>
     <t>Pant</t>
   </si>
   <si>
@@ -201,21 +219,45 @@
     <t>D:\PICS\FTP\ALEX</t>
   </si>
   <si>
+    <t>E:\Pluie\PICS\ALEX</t>
+  </si>
+  <si>
     <t>MFINRAE</t>
   </si>
   <si>
     <t>antilope_j1_000015_</t>
   </si>
   <si>
+    <t>D:\PICS\FTP\11_Antilope_1h_J+1_desag15min_avec_panthere</t>
+  </si>
+  <si>
+    <t>E:\Pluie\PICS\11_Antilope_1h_J+1_desag15min_avec_panthere</t>
+  </si>
+  <si>
     <t>MF_Cerema</t>
   </si>
   <si>
     <t>ANTILOPE_Cerema_TD_</t>
   </si>
   <si>
+    <t>D:\PICS\FTP\12_Antilope_MFCerema_15min_Tdiff_ProjMF</t>
+  </si>
+  <si>
+    <t>E:\Pluie\PICS\12_Antilope_MFCerema_15min_Tdiff_ProjMF</t>
+  </si>
+  <si>
+    <t>D:\PICS\FTP\12_Antilope_MFCerema_15min_Tdiff_ProjMF_201410</t>
+  </si>
+  <si>
+    <t>E:\Pluie\PICS\12_Antilope_MFCerema_15min_Tdiff_ProjMF_201410</t>
+  </si>
+  <si>
     <t>D:\PICS\FTP\LABATUT LAURENT\20140928_20140930</t>
   </si>
   <si>
+    <t>E:\Pluie\PICS\LABATUT LAURENT\20140928_20140930</t>
+  </si>
+  <si>
     <t>Nimes</t>
   </si>
   <si>
@@ -237,6 +279,9 @@
     <t>D:\jobfred\lames_eau_Vistre_Aval\2002</t>
   </si>
   <si>
+    <t>D:\Nabil\Pluie_nimes\_Cerema_Pluie\Data\lames_eau_Vistre_Aval\2002</t>
+  </si>
+  <si>
     <t>Z1</t>
   </si>
   <si>
@@ -249,18 +294,72 @@
     <t>D:\jobfred\lames_eau_Vistre_Aval\2005</t>
   </si>
   <si>
+    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2005</t>
+  </si>
+  <si>
+    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\200509</t>
+  </si>
+  <si>
     <t>C:\Cartino2D\_Pluie\lames_eau_Vistre_Aval\2014</t>
   </si>
   <si>
     <t>D:\jobfred\lames_eau_Vistre_Aval\2014</t>
   </si>
   <si>
+    <t>C:\Cartino2D\_Pluie\lames_eau_Vistre_Aval\2015</t>
+  </si>
+  <si>
+    <t>D:\jobfred\lames_eau_Vistre_Aval\2015</t>
+  </si>
+  <si>
+    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2015</t>
+  </si>
+  <si>
+    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2016</t>
+  </si>
+  <si>
     <t>C:\Cartino2D\_Pluie\lames_eau_Vistre_Aval\2021</t>
   </si>
   <si>
     <t>D:\jobfred\lames_eau_Vistre_Aval\2021</t>
   </si>
   <si>
+    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2021</t>
+  </si>
+  <si>
+    <t>PANTHERE_</t>
+  </si>
+  <si>
+    <t>%d_%m_%Y %H_%M</t>
+  </si>
+  <si>
+    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\Panthere_grille_asc_2016</t>
+  </si>
+  <si>
+    <t>Z3</t>
+  </si>
+  <si>
+    <t>GR_Z3_</t>
+  </si>
+  <si>
+    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\102021</t>
+  </si>
+  <si>
+    <t>Guadeloupe</t>
+  </si>
+  <si>
+    <t>ProjMF_Evt_Fiona_15min_CEREMA</t>
+  </si>
+  <si>
+    <t>_15min_cerema</t>
+  </si>
+  <si>
+    <t>ANTILOPE_PRECIP_</t>
+  </si>
+  <si>
+    <t>D:\Nabil\FIONA\Cerema20230616</t>
+  </si>
+  <si>
     <t>SHYREG</t>
   </si>
   <si>
@@ -291,109 +390,55 @@
     <t>D:\jobfred\SHYREG_2018_27583</t>
   </si>
   <si>
+    <t>D:\Nabil\Pluie_nimes\_Cerema_Pluie\Data\SHYREG_2018_27583</t>
+  </si>
+  <si>
     <t>D:\jobfred\SHYREG_2018_ProjMF</t>
   </si>
   <si>
-    <t>Nabil</t>
-  </si>
-  <si>
-    <t>C:\Cartino2D\_Pluie\lames_eau_Vistre_Aval\2015</t>
-  </si>
-  <si>
-    <t>D:\jobfred\lames_eau_Vistre_Aval\2015</t>
-  </si>
-  <si>
-    <t>Z3</t>
-  </si>
-  <si>
-    <t>GR_Z3_</t>
-  </si>
-  <si>
-    <t>Guadeloupe</t>
-  </si>
-  <si>
-    <t>ProjMF_Evt_Fiona_15min_CEREMA</t>
-  </si>
-  <si>
-    <t>ANTILOPE_PRECIP_</t>
-  </si>
-  <si>
-    <t>_15min_cerema</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2016</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2021</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\102021</t>
-  </si>
-  <si>
-    <t>D:\Nabil\FIONA\Cerema20230616</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2015</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2014</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\200509</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2005</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Pluie_nimes\_Cerema_Pluie\Data\lames_eau_Vistre_Aval\2002</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Pluie_nimes\_Cerema_Pluie\Data\SHYREG_2018_27583</t>
-  </si>
-  <si>
-    <t>PANTHERE_</t>
-  </si>
-  <si>
-    <t>D:\Nabil\Nimes\lames_eau_Vistre_Aval\Panthere_grille_asc_2016</t>
-  </si>
-  <si>
-    <t>E:\Pluie\PICS\LABATUT LAURENT\20140928_20140930</t>
-  </si>
-  <si>
-    <t>E:\Pluie\PICS\envoiMF09062021\05_Antilope_1h_J+1</t>
-  </si>
-  <si>
-    <t>E:\Pluie\PICS\envoiMF09062021\03_Antilope_15min_Tdiff</t>
-  </si>
-  <si>
-    <t>E:\Pluie\PICS\envoiMF09062021\08_Antilope_15min_Tdiff_inter</t>
-  </si>
-  <si>
-    <t>E:\Pluie\PICS\ALEX</t>
-  </si>
-  <si>
-    <t>D:\PICS\FTP\11_Antilope_1h_J+1_desag15min_avec_panthere</t>
-  </si>
-  <si>
-    <t>D:\PICS\FTP\12_Antilope_MFCerema_15min_Tdiff_ProjMF</t>
-  </si>
-  <si>
-    <t>E:\Pluie\PICS\11_Antilope_1h_J+1_desag15min_avec_panthere</t>
-  </si>
-  <si>
-    <t>E:\Pluie\PICS\12_Antilope_MFCerema_15min_Tdiff_ProjMF</t>
-  </si>
-  <si>
-    <t>D:\PICS\FTP\12_Antilope_MFCerema_15min_Tdiff_ProjMF_201410</t>
-  </si>
-  <si>
-    <t>E:\Pluie\PICS\12_Antilope_MFCerema_15min_Tdiff_ProjMF_201410</t>
-  </si>
-  <si>
-    <t>Formatdate</t>
-  </si>
-  <si>
-    <t>%d_%m_%Y %H_%M</t>
+    <t>GERS</t>
+  </si>
+  <si>
+    <t>C:\PROJET\2024_GERS\LAMEDO\ANTILOPEJ1</t>
+  </si>
+  <si>
+    <t>C:\Cartino2D\France\_Pluie\INRAE\2014</t>
+  </si>
+  <si>
+    <t>RESTONICA</t>
+  </si>
+  <si>
+    <t>C:\Cartino2D\France\_Pluie\Data\AntilopeJ1_restonica_nov_2023</t>
+  </si>
+  <si>
+    <t>C:\Cartino2D\France\_Pluie\Data\Antilope15_restonica_nov_2023</t>
+  </si>
+  <si>
+    <t>Garance</t>
+  </si>
+  <si>
+    <t>C:\Cartino2D\France\_Pluie\Data\ANTILOPE_PP_GARANCE_20250228</t>
+  </si>
+  <si>
+    <t>RancureAsse</t>
+  </si>
+  <si>
+    <t>C:\Pluie_Asse\16_12_2019_panthere_corrige</t>
+  </si>
+  <si>
+    <t>C:\Pluie_Asse\19_11_2019_panthere_corrige</t>
+  </si>
+  <si>
+    <t>C:\Pluie_Asse\20_10_2019_panthere_corrige</t>
+  </si>
+  <si>
+    <t>C:\Pluie_Asse\25_10_2018_panthere_corrige</t>
+  </si>
+  <si>
+    <t>C:\Cartino2D\07_03_2018_panthere_corrige</t>
+  </si>
+  <si>
+    <t>F:\Cartino2D\France\_Pluie\2014</t>
   </si>
 </sst>
 </file>
@@ -407,18 +452,14 @@
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF4472C4"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -431,13 +472,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor rgb="FFC0C0C0"/>
+        <bgColor indexed="22"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFF9900"/>
+        <bgColor indexed="52"/>
       </patternFill>
     </fill>
   </fills>
@@ -455,10 +496,10 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -472,74 +513,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF4472C4"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF92D050"/>
-      <rgbColor rgb="FFFFC000"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -594,108 +567,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -703,7 +582,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -729,7 +608,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -781,16 +660,28 @@
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -806,7 +697,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -838,73 +729,68 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:X37"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125"/>
-    <col min="3" max="3" width="6.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625"/>
+    <col min="3" max="3" width="6.88671875" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" customWidth="1"/>
-    <col min="6" max="6" width="38.140625" customWidth="1"/>
-    <col min="7" max="7" width="78.42578125" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" customWidth="1"/>
-    <col min="9" max="9" width="18.5703125" customWidth="1"/>
-    <col min="10" max="10" width="27.7109375" customWidth="1"/>
-    <col min="11" max="12" width="9.42578125" customWidth="1"/>
-    <col min="13" max="13" width="5.85546875" customWidth="1"/>
-    <col min="14" max="14" width="3.7109375" customWidth="1"/>
-    <col min="15" max="15" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" customWidth="1"/>
+    <col min="6" max="6" width="38.109375" customWidth="1"/>
+    <col min="7" max="7" width="78.44140625" customWidth="1"/>
+    <col min="8" max="8" width="9.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.5546875" customWidth="1"/>
+    <col min="10" max="10" width="27.6640625" customWidth="1"/>
+    <col min="11" max="12" width="9.44140625" customWidth="1"/>
+    <col min="13" max="13" width="5.88671875" customWidth="1"/>
+    <col min="14" max="14" width="3.6640625" customWidth="1"/>
+    <col min="15" max="15" width="10.6640625" customWidth="1"/>
     <col min="16" max="16" width="10" customWidth="1"/>
-    <col min="17" max="17" width="7.28515625" customWidth="1"/>
-    <col min="18" max="19" width="16.5703125" customWidth="1"/>
-    <col min="20" max="20" width="8.7109375" customWidth="1"/>
-    <col min="21" max="21" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="74.42578125" customWidth="1"/>
-    <col min="23" max="23" width="78.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="56.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="1026" width="10.7109375" customWidth="1"/>
+    <col min="17" max="17" width="7.33203125" customWidth="1"/>
+    <col min="18" max="19" width="16.5546875" customWidth="1"/>
+    <col min="20" max="20" width="8.6640625" customWidth="1"/>
+    <col min="21" max="21" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="74.44140625" customWidth="1"/>
+    <col min="23" max="23" width="78.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="56.5546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="1026" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -913,69 +799,69 @@
       <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="V1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F2" t="str">
         <f t="shared" ref="F2:F27" si="0">_xlfn.CONCAT(Q2,"_",T2,"_",B2,"_",N2,O2,"_",D2,"_",E2,"_",C2)</f>
         <v>27572_Evt_Anti_60min_J0_Schapi_</v>
       </c>
       <c r="G2" t="str">
-        <f>W2</f>
+        <f t="shared" ref="G2:G9" si="1">W2</f>
         <v>D:\jobfred\2_cas1_ANTILOPE_1h_Schapi</v>
       </c>
       <c r="H2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -990,10 +876,10 @@
         <v>60</v>
       </c>
       <c r="O2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q2">
         <v>27572</v>
@@ -1005,41 +891,41 @@
         <v>100</v>
       </c>
       <c r="T2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="W2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F3" t="str">
         <f t="shared" si="0"/>
         <v>2154_Evt_Anti_60min_J1_Schapi_</v>
       </c>
       <c r="G3" t="str">
-        <f>W3</f>
+        <f t="shared" si="1"/>
         <v>D:\jobfred\2_cas2_ANTILOPE_J1_1h_Schapi</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K3">
         <v>2</v>
@@ -1054,10 +940,10 @@
         <v>60</v>
       </c>
       <c r="O3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q3">
         <v>2154</v>
@@ -1069,38 +955,38 @@
         <v>100</v>
       </c>
       <c r="T3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="W3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" si="0"/>
         <v>2154_Evt_Anti_60min_J2_PluginQgis_</v>
       </c>
       <c r="G4" t="str">
-        <f>W4</f>
+        <f t="shared" si="1"/>
         <v>D:\jobfred\2_cas3_ANTJ1_MPL_pluginQgis</v>
       </c>
       <c r="H4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -1115,10 +1001,10 @@
         <v>60</v>
       </c>
       <c r="O4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q4">
         <v>2154</v>
@@ -1130,41 +1016,41 @@
         <v>100</v>
       </c>
       <c r="T4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="W4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="0"/>
         <v>4326_Evt_Anti_60min_J3_MF_</v>
       </c>
       <c r="G5" t="str">
-        <f>W5</f>
+        <f t="shared" si="1"/>
         <v>E:\Pluie\PICS\envoiMF09062021\05_Antilope_1h_J+1</v>
       </c>
       <c r="H5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -1179,10 +1065,10 @@
         <v>60</v>
       </c>
       <c r="O5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q5">
         <v>4326</v>
@@ -1191,41 +1077,41 @@
         <v>1E-3</v>
       </c>
       <c r="T5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="W5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" t="str">
         <f t="shared" si="0"/>
         <v>4326_Evt_Anti_15min_J4_MF_</v>
       </c>
       <c r="G6" t="str">
-        <f>W6</f>
+        <f t="shared" si="1"/>
         <v>E:\Pluie\PICS\envoiMF09062021\03_Antilope_15min_Tdiff</v>
       </c>
       <c r="H6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="K6">
         <v>1</v>
@@ -1240,10 +1126,10 @@
         <v>15</v>
       </c>
       <c r="O6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q6">
         <v>4326</v>
@@ -1252,41 +1138,41 @@
         <v>1E-3</v>
       </c>
       <c r="T6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="W6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F7" t="str">
         <f t="shared" si="0"/>
         <v>ProjMF_Evt_Anti_15min_J5_MF_</v>
       </c>
       <c r="G7" t="str">
-        <f>W7</f>
+        <f t="shared" si="1"/>
         <v>E:\Pluie\PICS\envoiMF09062021\08_Antilope_15min_Tdiff_inter</v>
       </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J7" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="K7">
         <v>1</v>
@@ -1301,13 +1187,13 @@
         <v>15</v>
       </c>
       <c r="O7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R7" s="4">
         <v>1092.843190094</v>
@@ -1316,41 +1202,41 @@
         <v>109.28431900939999</v>
       </c>
       <c r="T7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="W7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F8" t="str">
         <f t="shared" si="0"/>
         <v>2154_Evt_Pant_5min_J0_Schapi_</v>
       </c>
       <c r="G8" t="str">
-        <f>W8</f>
+        <f t="shared" si="1"/>
         <v>D:\jobfred\1_PANTHERE_5min</v>
       </c>
       <c r="H8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J8" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="K8">
         <v>2</v>
@@ -1365,10 +1251,10 @@
         <v>5</v>
       </c>
       <c r="O8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q8">
         <v>2154</v>
@@ -1380,41 +1266,41 @@
         <v>100</v>
       </c>
       <c r="T8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V8" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="W8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F9" t="str">
         <f t="shared" si="0"/>
         <v>ProjMF_Evt_Anti_60min_JALEX_MF_</v>
       </c>
       <c r="G9" t="str">
-        <f>W9</f>
+        <f t="shared" si="1"/>
         <v>E:\Pluie\PICS\ALEX</v>
       </c>
       <c r="H9" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="K9">
         <v>1</v>
@@ -1429,13 +1315,13 @@
         <v>60</v>
       </c>
       <c r="O9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R9" s="4">
         <v>1092.843190094</v>
@@ -1444,41 +1330,41 @@
         <v>109.28431900939999</v>
       </c>
       <c r="T9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="W9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F10" t="str">
         <f t="shared" si="0"/>
         <v>2154_Evt_Anti_15min_J1_MFINRAE_</v>
       </c>
       <c r="G10" t="str">
-        <f>W10</f>
+        <f t="shared" ref="G10:G13" si="2">W10</f>
         <v>E:\Pluie\PICS\11_Antilope_1h_J+1_desag15min_avec_panthere</v>
       </c>
       <c r="H10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J10" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -1493,10 +1379,10 @@
         <v>15</v>
       </c>
       <c r="O10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q10">
         <v>2154</v>
@@ -1508,41 +1394,41 @@
         <v>100</v>
       </c>
       <c r="T10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V10" t="s">
-        <v>113</v>
+        <v>64</v>
       </c>
       <c r="W10" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F11" t="str">
         <f t="shared" si="0"/>
         <v>ProjMF_Evt_Anti_15min_J1_MF_Cerema_</v>
       </c>
       <c r="G11" t="str">
-        <f>W11</f>
+        <f t="shared" si="2"/>
         <v>E:\Pluie\PICS\12_Antilope_MFCerema_15min_Tdiff_ProjMF</v>
       </c>
       <c r="H11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J11" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -1557,13 +1443,13 @@
         <v>15</v>
       </c>
       <c r="O11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q11" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R11" s="4">
         <v>1092.843190094</v>
@@ -1572,44 +1458,44 @@
         <v>109.28431900939999</v>
       </c>
       <c r="T11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V11" t="s">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="W11" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C12">
         <v>2014</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F12" t="str">
-        <f t="shared" ref="F12" si="1">_xlfn.CONCAT(Q12,"_",T12,"_",B12,"_",N12,O12,"_",D12,"_",E12,"_",C12)</f>
+        <f>_xlfn.CONCAT(Q12,"_",T12,"_",B12,"_",N12,O12,"_",D12,"_",E12,"_",C12)</f>
         <v>ProjMF_Evt_Anti_15min_J1_MF_Cerema_2014</v>
       </c>
       <c r="G12" t="str">
-        <f>W12</f>
+        <f t="shared" si="2"/>
         <v>E:\Pluie\PICS\12_Antilope_MFCerema_15min_Tdiff_ProjMF_201410</v>
       </c>
       <c r="H12" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J12" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="K12">
         <v>1</v>
@@ -1624,13 +1510,13 @@
         <v>15</v>
       </c>
       <c r="O12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q12" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R12" s="4">
         <v>1092.843190094</v>
@@ -1639,41 +1525,41 @@
         <v>109.28431900939999</v>
       </c>
       <c r="T12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V12" t="s">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="W12" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F13" t="str">
         <f t="shared" si="0"/>
         <v>ProjMF_Evt_Anti_60min_J1_MF_</v>
       </c>
       <c r="G13" t="str">
-        <f>W13</f>
+        <f t="shared" si="2"/>
         <v>E:\Pluie\PICS\LABATUT LAURENT\20140928_20140930</v>
       </c>
       <c r="H13" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J13" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="K13">
         <v>1</v>
@@ -1688,13 +1574,13 @@
         <v>60</v>
       </c>
       <c r="O13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q13" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R13" s="4">
         <v>1092.843190094</v>
@@ -1703,44 +1589,44 @@
         <v>109.28431900939999</v>
       </c>
       <c r="T13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V13" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="W13" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C14">
         <v>2002</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F14" t="str">
         <f t="shared" si="0"/>
         <v>27583_Evt_Nimes_5min_Z2_NIMES_2002</v>
       </c>
       <c r="G14" t="str">
-        <f>W14</f>
-        <v>D:\jobfred\lames_eau_Vistre_Aval\2002</v>
+        <f>X14</f>
+        <v>D:\Nabil\Pluie_nimes\_Cerema_Pluie\Data\lames_eau_Vistre_Aval\2002</v>
       </c>
       <c r="H14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J14" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="K14">
         <v>1</v>
@@ -1755,10 +1641,10 @@
         <v>5</v>
       </c>
       <c r="O14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P14" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q14">
         <v>27583</v>
@@ -1770,47 +1656,47 @@
         <v>50</v>
       </c>
       <c r="T14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V14" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="W14" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="X14" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C15">
         <v>2005</v>
       </c>
       <c r="D15" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="E15" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F15" t="str">
         <f t="shared" si="0"/>
         <v>27583_Evt_Nimes_5min_Z1_NIMES_2005</v>
       </c>
       <c r="G15" t="str">
-        <f>W15</f>
-        <v>D:\jobfred\lames_eau_Vistre_Aval\2005</v>
+        <f t="shared" ref="G15:G20" si="3">X15</f>
+        <v>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2005</v>
       </c>
       <c r="H15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J15" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="K15">
         <v>1</v>
@@ -1825,10 +1711,10 @@
         <v>5</v>
       </c>
       <c r="O15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P15" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q15">
         <v>27583</v>
@@ -1840,47 +1726,47 @@
         <v>50</v>
       </c>
       <c r="T15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V15" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="W15" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="X15" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C16">
         <v>2005</v>
       </c>
       <c r="D16" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E16" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F16" t="str">
         <f>_xlfn.CONCAT(Q16,"_",T16,"_",B16,"_",N16,O16,"_",D16,"_",E16,"_",C16)</f>
         <v>27583_Evt_Nimes_5min_Z2_NIMES_2005</v>
       </c>
       <c r="G16" t="str">
-        <f>W16</f>
-        <v>D:\jobfred\lames_eau_Vistre_Aval\2005</v>
+        <f t="shared" si="3"/>
+        <v>D:\Nabil\Nimes\lames_eau_Vistre_Aval\200509</v>
       </c>
       <c r="H16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J16" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="K16">
         <v>1</v>
@@ -1895,10 +1781,10 @@
         <v>5</v>
       </c>
       <c r="O16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P16" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q16">
         <v>27583</v>
@@ -1910,47 +1796,47 @@
         <v>50</v>
       </c>
       <c r="T16" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V16" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="W16" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="X16" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C17">
         <v>2014</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E17" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F17" t="str">
         <f t="shared" si="0"/>
         <v>27583_Evt_Nimes_5min_Z2_NIMES_2014</v>
       </c>
       <c r="G17" t="str">
-        <f>W17</f>
-        <v>D:\jobfred\lames_eau_Vistre_Aval\2014</v>
+        <f t="shared" si="3"/>
+        <v>F:\Cartino2D\France\_Pluie\2014</v>
       </c>
       <c r="H17" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J17" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="K17">
         <v>1</v>
@@ -1965,10 +1851,10 @@
         <v>5</v>
       </c>
       <c r="O17" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P17" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q17">
         <v>27583</v>
@@ -1980,47 +1866,47 @@
         <v>50</v>
       </c>
       <c r="T17" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V17" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="W17" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="X17" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C18">
         <v>2015</v>
       </c>
       <c r="D18" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E18" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F18" t="str">
         <f t="shared" si="0"/>
         <v>27583_Evt_Nimes_5min_Z2_NIMES_2015</v>
       </c>
       <c r="G18" t="str">
-        <f>W18</f>
-        <v>D:\jobfred\lames_eau_Vistre_Aval\2015</v>
+        <f t="shared" si="3"/>
+        <v>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2015</v>
       </c>
       <c r="H18" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J18" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -2035,10 +1921,10 @@
         <v>5</v>
       </c>
       <c r="O18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P18" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q18">
         <v>27583</v>
@@ -2050,47 +1936,47 @@
         <v>50</v>
       </c>
       <c r="T18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V18" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="W18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="X18" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C19">
         <v>2016</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F19" t="str">
-        <f>_xlfn.CONCAT(Q19,"_",T19,"_",B19,"_",N19,O19,"_",D19,"_",E19,"_",C19)</f>
+        <f t="shared" ref="F19:F22" si="4">_xlfn.CONCAT(Q19,"_",T19,"_",B19,"_",N19,O19,"_",D19,"_",E19,"_",C19)</f>
         <v>27583_Evt_Nimes_5min_Z2_NIMES_2016</v>
       </c>
       <c r="G19" t="str">
-        <f>W19</f>
-        <v>D:\jobfred\lames_eau_Vistre_Aval\2015</v>
+        <f t="shared" si="3"/>
+        <v>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2016</v>
       </c>
       <c r="H19" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J19" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="K19">
         <v>1</v>
@@ -2105,10 +1991,10 @@
         <v>5</v>
       </c>
       <c r="O19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P19" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q19">
         <v>27583</v>
@@ -2120,47 +2006,47 @@
         <v>50</v>
       </c>
       <c r="T19" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="W19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="X19" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C20">
         <v>2021</v>
       </c>
       <c r="D20" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E20" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F20" t="str">
-        <f>_xlfn.CONCAT(Q20,"_",T20,"_",B20,"_",N20,O20,"_",D20,"_",E20,"_",C20)</f>
+        <f t="shared" si="4"/>
         <v>27583_Evt_Nimes_5min_Z2_NIMES_2021</v>
       </c>
       <c r="G20" t="str">
-        <f>W20</f>
-        <v>D:\jobfred\lames_eau_Vistre_Aval\2021</v>
+        <f t="shared" si="3"/>
+        <v>D:\Nabil\Nimes\lames_eau_Vistre_Aval\2021</v>
       </c>
       <c r="H20" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J20" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="K20">
         <v>1</v>
@@ -2175,10 +2061,10 @@
         <v>5</v>
       </c>
       <c r="O20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P20" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q20">
         <v>27583</v>
@@ -2190,36 +2076,36 @@
         <v>50</v>
       </c>
       <c r="T20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V20" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="W20" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="X20" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C21">
         <v>2016</v>
       </c>
       <c r="D21" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F21" t="str">
-        <f>_xlfn.CONCAT(Q21,"_",T21,"_",B21,"_",N21,O21,"_",D21,"_",E21,"_",C21)</f>
+        <f t="shared" si="4"/>
         <v>2154_Evt_Nimes_5min_Z2_MF_2016</v>
       </c>
       <c r="G21" t="str">
@@ -2227,10 +2113,10 @@
         <v>D:\Nabil\Nimes\lames_eau_Vistre_Aval\Panthere_grille_asc_2016</v>
       </c>
       <c r="H21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J21" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="K21">
         <v>1</v>
@@ -2245,10 +2131,10 @@
         <v>5</v>
       </c>
       <c r="O21" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P21" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q21">
         <v>2154</v>
@@ -2260,44 +2146,44 @@
         <v>100</v>
       </c>
       <c r="T21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="U21" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="X21" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="C22">
         <v>2021</v>
       </c>
       <c r="D22" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E22" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F22" t="str">
-        <f>_xlfn.CONCAT(Q22,"_",T22,"_",B22,"_",N22,O22,"_",D22,"_",E22,"_",C22)</f>
+        <f t="shared" si="4"/>
         <v>27583_Evt_Nimes_5min_Z3_NIMES_2021</v>
       </c>
       <c r="G22" t="str">
-        <f>W22</f>
+        <f t="shared" ref="G22:G27" si="5">W22</f>
         <v>D:\jobfred\lames_eau_Vistre_Aval\2021</v>
       </c>
       <c r="H22" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J22" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="K22">
         <v>1</v>
@@ -2312,10 +2198,10 @@
         <v>5</v>
       </c>
       <c r="O22" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P22" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q22">
         <v>27583</v>
@@ -2327,49 +2213,49 @@
         <v>50</v>
       </c>
       <c r="T22" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="V22" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="W22" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="X22" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="C23">
         <v>2022</v>
       </c>
       <c r="D23" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E23" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F23" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="G23">
-        <f>W23</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="H23" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I23" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="J23" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="K23">
         <v>1</v>
@@ -2384,13 +2270,13 @@
         <v>15</v>
       </c>
       <c r="O23" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P23" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q23" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R23">
         <v>1000</v>
@@ -2399,13 +2285,13 @@
         <v>100</v>
       </c>
       <c r="T23" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="X23" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>99</v>
       </c>
@@ -2414,36 +2300,36 @@
         <v>______</v>
       </c>
       <c r="G24">
-        <f>W24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="D25" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="E25" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="F25" t="str">
         <f t="shared" si="0"/>
         <v>2154_Stat_SHYREG_-99min_RR_INRAE_</v>
       </c>
       <c r="G25" t="str">
-        <f>W25</f>
+        <f t="shared" si="5"/>
         <v>D:\jobfred\SHYREG_2018_2154</v>
       </c>
       <c r="H25" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J25" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
       <c r="K25">
         <v>0</v>
@@ -2455,10 +2341,10 @@
         <v>-99</v>
       </c>
       <c r="O25" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q25">
         <v>2154</v>
@@ -2470,41 +2356,41 @@
         <v>100</v>
       </c>
       <c r="T25" t="s">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="V25" t="s">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="W25" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="D26" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="E26" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="F26" t="str">
         <f t="shared" si="0"/>
         <v>27583_Stat_SHYREG_-99min_RR_INRAE_</v>
       </c>
       <c r="G26" t="str">
-        <f>W26</f>
+        <f t="shared" si="5"/>
         <v>D:\jobfred\SHYREG_2018_27583</v>
       </c>
       <c r="H26" t="s">
-        <v>83</v>
+        <v>115</v>
       </c>
       <c r="J26" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -2516,10 +2402,10 @@
         <v>-99</v>
       </c>
       <c r="O26" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P26" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q26">
         <v>27583</v>
@@ -2531,44 +2417,44 @@
         <v>50</v>
       </c>
       <c r="T26" t="s">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="V26" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="W26" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="X26" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="D27" t="s">
-        <v>77</v>
+        <v>109</v>
       </c>
       <c r="E27" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="F27" t="str">
         <f t="shared" si="0"/>
         <v>ProjMF_Stat_SHYREG_-99min_RR_INRAE_</v>
       </c>
       <c r="G27" t="str">
-        <f>W27</f>
+        <f t="shared" si="5"/>
         <v>D:\jobfred\SHYREG_2018_ProjMF</v>
       </c>
       <c r="H27" t="s">
-        <v>83</v>
+        <v>115</v>
       </c>
       <c r="J27" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
       <c r="K27">
         <v>0</v>
@@ -2580,13 +2466,13 @@
         <v>-99</v>
       </c>
       <c r="O27" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="P27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="Q27" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="R27" s="4">
         <v>1092.843190094</v>
@@ -2595,10 +2481,586 @@
         <v>109.28431900939999</v>
       </c>
       <c r="T27" t="s">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="W27" t="s">
-        <v>86</v>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>22</v>
+      </c>
+      <c r="B28" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28">
+        <v>2014</v>
+      </c>
+      <c r="D28" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" t="s">
+        <v>41</v>
+      </c>
+      <c r="F28" t="str">
+        <f t="shared" ref="F28:F32" si="6">_xlfn.CONCAT(Q28,"_",T28,"_",B28,"_",N28,O28,"_",D28,"_",E28,"_",C28)</f>
+        <v>2154_Evt_GERS_60min_J1_MF_2014</v>
+      </c>
+      <c r="G28" t="s">
+        <v>121</v>
+      </c>
+      <c r="H28" t="s">
+        <v>38</v>
+      </c>
+      <c r="K28">
+        <v>1</v>
+      </c>
+      <c r="L28">
+        <v>12</v>
+      </c>
+      <c r="M28">
+        <v>10</v>
+      </c>
+      <c r="N28">
+        <v>60</v>
+      </c>
+      <c r="O28" t="s">
+        <v>29</v>
+      </c>
+      <c r="P28" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q28">
+        <v>2154</v>
+      </c>
+      <c r="R28">
+        <v>1000</v>
+      </c>
+      <c r="S28">
+        <v>100</v>
+      </c>
+      <c r="T28" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>23</v>
+      </c>
+      <c r="B29" t="s">
+        <v>120</v>
+      </c>
+      <c r="C29">
+        <v>2014</v>
+      </c>
+      <c r="D29" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" t="s">
+        <v>110</v>
+      </c>
+      <c r="F29" t="str">
+        <f t="shared" si="6"/>
+        <v>2154_Evt_GERS_15min_J1_INRAE_2014</v>
+      </c>
+      <c r="G29" t="s">
+        <v>122</v>
+      </c>
+      <c r="H29" t="s">
+        <v>27</v>
+      </c>
+      <c r="J29" t="s">
+        <v>63</v>
+      </c>
+      <c r="K29">
+        <v>2</v>
+      </c>
+      <c r="L29">
+        <v>12</v>
+      </c>
+      <c r="M29">
+        <v>1</v>
+      </c>
+      <c r="N29">
+        <v>15</v>
+      </c>
+      <c r="O29" t="s">
+        <v>29</v>
+      </c>
+      <c r="P29" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q29">
+        <v>2154</v>
+      </c>
+      <c r="R29">
+        <v>1000</v>
+      </c>
+      <c r="S29">
+        <v>100</v>
+      </c>
+      <c r="T29" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>24</v>
+      </c>
+      <c r="B30" t="s">
+        <v>123</v>
+      </c>
+      <c r="C30">
+        <v>2023</v>
+      </c>
+      <c r="D30" t="s">
+        <v>33</v>
+      </c>
+      <c r="E30" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" t="str">
+        <f t="shared" si="6"/>
+        <v>2154_Evt_RESTONICA_60min_J1_MF_2023</v>
+      </c>
+      <c r="G30" t="s">
+        <v>124</v>
+      </c>
+      <c r="H30" t="s">
+        <v>38</v>
+      </c>
+      <c r="K30">
+        <v>1</v>
+      </c>
+      <c r="L30">
+        <v>12</v>
+      </c>
+      <c r="M30">
+        <v>10</v>
+      </c>
+      <c r="N30">
+        <v>60</v>
+      </c>
+      <c r="O30" t="s">
+        <v>29</v>
+      </c>
+      <c r="P30" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q30">
+        <v>2154</v>
+      </c>
+      <c r="R30">
+        <v>1000</v>
+      </c>
+      <c r="S30">
+        <v>100</v>
+      </c>
+      <c r="T30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>25</v>
+      </c>
+      <c r="B31" t="s">
+        <v>123</v>
+      </c>
+      <c r="C31">
+        <v>2023</v>
+      </c>
+      <c r="D31" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" t="s">
+        <v>41</v>
+      </c>
+      <c r="F31" t="str">
+        <f t="shared" si="6"/>
+        <v>2154_Evt_RESTONICA_15min_J0_MF_2023</v>
+      </c>
+      <c r="G31" t="s">
+        <v>125</v>
+      </c>
+      <c r="H31" t="s">
+        <v>38</v>
+      </c>
+      <c r="K31">
+        <v>1</v>
+      </c>
+      <c r="L31">
+        <v>12</v>
+      </c>
+      <c r="M31">
+        <v>10</v>
+      </c>
+      <c r="N31">
+        <v>15</v>
+      </c>
+      <c r="O31" t="s">
+        <v>29</v>
+      </c>
+      <c r="P31" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q31">
+        <v>2154</v>
+      </c>
+      <c r="R31">
+        <v>1000</v>
+      </c>
+      <c r="S31">
+        <v>100</v>
+      </c>
+      <c r="T31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>26</v>
+      </c>
+      <c r="B32" t="s">
+        <v>126</v>
+      </c>
+      <c r="C32">
+        <v>2025</v>
+      </c>
+      <c r="D32" t="s">
+        <v>33</v>
+      </c>
+      <c r="E32" t="s">
+        <v>41</v>
+      </c>
+      <c r="F32" t="str">
+        <f t="shared" si="6"/>
+        <v>2975_Evt_Garance_15min_J1_MF_2025</v>
+      </c>
+      <c r="G32" t="s">
+        <v>127</v>
+      </c>
+      <c r="H32" t="s">
+        <v>27</v>
+      </c>
+      <c r="J32" t="s">
+        <v>63</v>
+      </c>
+      <c r="K32">
+        <v>2</v>
+      </c>
+      <c r="L32">
+        <v>12</v>
+      </c>
+      <c r="M32">
+        <v>1</v>
+      </c>
+      <c r="N32">
+        <v>15</v>
+      </c>
+      <c r="O32" t="s">
+        <v>29</v>
+      </c>
+      <c r="P32" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q32">
+        <v>2975</v>
+      </c>
+      <c r="R32">
+        <v>1000</v>
+      </c>
+      <c r="S32">
+        <v>100</v>
+      </c>
+      <c r="T32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>27</v>
+      </c>
+      <c r="B33" t="s">
+        <v>128</v>
+      </c>
+      <c r="C33">
+        <v>201803</v>
+      </c>
+      <c r="D33" t="s">
+        <v>33</v>
+      </c>
+      <c r="E33" t="s">
+        <v>41</v>
+      </c>
+      <c r="F33" t="str">
+        <f t="shared" ref="F33" si="7">_xlfn.CONCAT(Q33,"_",T33,"_",B33,"_",N33,O33,"_",D33,"_",E33,"_",C33)</f>
+        <v>2154_Evt_RancureAsse_15min_J1_MF_201803</v>
+      </c>
+      <c r="G33" t="s">
+        <v>133</v>
+      </c>
+      <c r="H33" t="s">
+        <v>27</v>
+      </c>
+      <c r="K33">
+        <v>1</v>
+      </c>
+      <c r="L33">
+        <v>12</v>
+      </c>
+      <c r="M33">
+        <v>1</v>
+      </c>
+      <c r="N33">
+        <v>15</v>
+      </c>
+      <c r="O33" t="s">
+        <v>29</v>
+      </c>
+      <c r="P33" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q33">
+        <v>2154</v>
+      </c>
+      <c r="R33">
+        <v>1000</v>
+      </c>
+      <c r="S33">
+        <v>100</v>
+      </c>
+      <c r="T33" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>28</v>
+      </c>
+      <c r="B34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34">
+        <v>201912</v>
+      </c>
+      <c r="D34" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" t="s">
+        <v>41</v>
+      </c>
+      <c r="F34" t="str">
+        <f t="shared" ref="F34" si="8">_xlfn.CONCAT(Q34,"_",T34,"_",B34,"_",N34,O34,"_",D34,"_",E34,"_",C34)</f>
+        <v>2154_Evt_RancureAsse_15min_J1_MF_201912</v>
+      </c>
+      <c r="G34" t="s">
+        <v>129</v>
+      </c>
+      <c r="H34" t="s">
+        <v>27</v>
+      </c>
+      <c r="K34">
+        <v>1</v>
+      </c>
+      <c r="L34">
+        <v>12</v>
+      </c>
+      <c r="M34">
+        <v>1</v>
+      </c>
+      <c r="N34">
+        <v>15</v>
+      </c>
+      <c r="O34" t="s">
+        <v>29</v>
+      </c>
+      <c r="P34" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q34">
+        <v>2154</v>
+      </c>
+      <c r="R34">
+        <v>1000</v>
+      </c>
+      <c r="S34">
+        <v>100</v>
+      </c>
+      <c r="T34" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>29</v>
+      </c>
+      <c r="B35" t="s">
+        <v>128</v>
+      </c>
+      <c r="C35">
+        <v>201911</v>
+      </c>
+      <c r="D35" t="s">
+        <v>33</v>
+      </c>
+      <c r="E35" t="s">
+        <v>41</v>
+      </c>
+      <c r="F35" t="str">
+        <f t="shared" ref="F35" si="9">_xlfn.CONCAT(Q35,"_",T35,"_",B35,"_",N35,O35,"_",D35,"_",E35,"_",C35)</f>
+        <v>2154_Evt_RancureAsse_15min_J1_MF_201911</v>
+      </c>
+      <c r="G35" t="s">
+        <v>130</v>
+      </c>
+      <c r="H35" t="s">
+        <v>27</v>
+      </c>
+      <c r="K35">
+        <v>1</v>
+      </c>
+      <c r="L35">
+        <v>12</v>
+      </c>
+      <c r="M35">
+        <v>1</v>
+      </c>
+      <c r="N35">
+        <v>15</v>
+      </c>
+      <c r="O35" t="s">
+        <v>29</v>
+      </c>
+      <c r="P35" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q35">
+        <v>2154</v>
+      </c>
+      <c r="R35">
+        <v>1000</v>
+      </c>
+      <c r="S35">
+        <v>100</v>
+      </c>
+      <c r="T35" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>30</v>
+      </c>
+      <c r="B36" t="s">
+        <v>128</v>
+      </c>
+      <c r="C36">
+        <v>201910</v>
+      </c>
+      <c r="D36" t="s">
+        <v>33</v>
+      </c>
+      <c r="E36" t="s">
+        <v>41</v>
+      </c>
+      <c r="F36" t="str">
+        <f t="shared" ref="F36" si="10">_xlfn.CONCAT(Q36,"_",T36,"_",B36,"_",N36,O36,"_",D36,"_",E36,"_",C36)</f>
+        <v>2154_Evt_RancureAsse_15min_J1_MF_201910</v>
+      </c>
+      <c r="G36" t="s">
+        <v>131</v>
+      </c>
+      <c r="H36" t="s">
+        <v>27</v>
+      </c>
+      <c r="K36">
+        <v>1</v>
+      </c>
+      <c r="L36">
+        <v>12</v>
+      </c>
+      <c r="M36">
+        <v>1</v>
+      </c>
+      <c r="N36">
+        <v>15</v>
+      </c>
+      <c r="O36" t="s">
+        <v>29</v>
+      </c>
+      <c r="P36" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q36">
+        <v>2154</v>
+      </c>
+      <c r="R36">
+        <v>1000</v>
+      </c>
+      <c r="S36">
+        <v>100</v>
+      </c>
+      <c r="T36" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>31</v>
+      </c>
+      <c r="B37" t="s">
+        <v>128</v>
+      </c>
+      <c r="C37">
+        <v>201810</v>
+      </c>
+      <c r="D37" t="s">
+        <v>33</v>
+      </c>
+      <c r="E37" t="s">
+        <v>41</v>
+      </c>
+      <c r="F37" t="str">
+        <f t="shared" ref="F37" si="11">_xlfn.CONCAT(Q37,"_",T37,"_",B37,"_",N37,O37,"_",D37,"_",E37,"_",C37)</f>
+        <v>2154_Evt_RancureAsse_15min_J1_MF_201810</v>
+      </c>
+      <c r="G37" t="s">
+        <v>132</v>
+      </c>
+      <c r="H37" t="s">
+        <v>27</v>
+      </c>
+      <c r="K37">
+        <v>1</v>
+      </c>
+      <c r="L37">
+        <v>12</v>
+      </c>
+      <c r="M37">
+        <v>1</v>
+      </c>
+      <c r="N37">
+        <v>15</v>
+      </c>
+      <c r="O37" t="s">
+        <v>29</v>
+      </c>
+      <c r="P37" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q37">
+        <v>2154</v>
+      </c>
+      <c r="R37">
+        <v>1000</v>
+      </c>
+      <c r="S37">
+        <v>100</v>
+      </c>
+      <c r="T37" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>